<commit_message>
Update BOM for Demoboard
</commit_message>
<xml_diff>
--- a/DemoBoard/inspireFly_PQ_payloadDemo_rev0.2.xlsx
+++ b/DemoBoard/inspireFly_PQ_payloadDemo_rev0.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shane\Documents\GitHub\Pocketqube-Payload-Boards\DemoBoard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A91C5ED8-2005-4152-BD2C-370892560E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153137ED-C548-4F63-8550-6DD4FB0EBDBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="2745" windowWidth="16200" windowHeight="9308" xr2:uid="{90A7F372-49DC-4743-8A39-617F3F98A630}"/>
+    <workbookView xWindow="2543" yWindow="2543" windowWidth="16200" windowHeight="9307" xr2:uid="{90A7F372-49DC-4743-8A39-617F3F98A630}"/>
   </bookViews>
   <sheets>
     <sheet name="Ordering Sheet" sheetId="1" r:id="rId1"/>
@@ -965,18 +965,18 @@
         <v>22</v>
       </c>
       <c r="D7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7">
         <f xml:space="preserve"> D7 *Constants!$C$1</f>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F7" s="4">
         <v>8.2000000000000003E-2</v>
       </c>
       <c r="G7" s="2">
         <f t="shared" si="0"/>
-        <v>1.23</v>
+        <v>1.6400000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="G26" s="2">
         <f>SUM(G2:G25)</f>
-        <v>82.294999999999987</v>
+        <v>82.704999999999984</v>
       </c>
     </row>
   </sheetData>

</xml_diff>